<commit_message>
Add connectivity-first weighting to the shortlist workbook
The Weights sheet now carries both weightings so the ranking can be switched by
copying one block into B8:B13.

Corrects a claim made in conversation: under connectivity-first weighting
Dhanbad stays #1 (4.00), Bhandara rises to #2 (3.80) rather than to #1, and
Akola falls from #2 to #5. Dhanbad is robust to the re-weighting because it wins
on fees, Hindi and rank-band fit simultaneously; the swap mainly separates
Bhandara (Nagpur ~60 km) from Akola (~250 km).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01C6PVtRwDf8eGQfJ9dqY3X7
</commit_message>
<xml_diff>
--- a/audit/aiq-privacy/mcc2026/AIQ_final_shortlist_criteria.xlsx
+++ b/audit/aiq-privacy/mcc2026/AIQ_final_shortlist_criteria.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -652,21 +652,95 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>NOTE: km and travel times are my estimates from public sources — verify before booking.</t>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Alternative: connectivity-first weighting (copy these into B8:B13 to switch)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NOTE: bond and PG-quota rules are revised annually. Confirm in the current counselling brochure.</t>
-        </is>
+          <t xml:space="preserve">   Info exposure</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Website staleness</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Connectivity</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Distance from Lucknow</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fees</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Hindi spoken</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Under connectivity-first: Dhanbad stays #1 (4.00), Bhandara rises to #2 (3.80), Akola drops from #2 to #5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NOTE: km and travel times are my estimates from public sources — verify before booking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NOTE: bond and PG-quota rules are revised annually. Confirm in the current counselling brochure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>NOTE: fees are state tuition estimates per year, excluding hostel/mess/caution deposits.</t>
         </is>

</xml_diff>